<commit_message>
update strategy definitions excel to inlcude LEP
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_wem_wam.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_wem_wam.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB4883C-6AFC-AB4B-993A-5AA8ED553102}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69F98C17-2246-6745-87E0-0E2B9FB378E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="36700" yWindow="2860" windowWidth="32100" windowHeight="19840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
     <sheet name="yaml" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$M$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$C$1:$N$65</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">yaml!$A$1:$D$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="734" uniqueCount="435">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="735" uniqueCount="436">
   <si>
     <t>subsector</t>
   </si>
@@ -1407,14 +1407,16 @@
   <si>
     <t>bulgaria_mitigation_action</t>
   </si>
+  <si>
+    <t>strategy_LEP</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0.0%"/>
   </numFmts>
   <fonts count="10" x14ac:knownFonts="1">
     <font>
@@ -1581,7 +1583,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="7" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1685,9 +1687,6 @@
     <xf numFmtId="4" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1696,9 +1695,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -2042,20 +2038,19 @@
     <col min="6" max="6" width="33.1640625" style="4" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="53.5" style="4" customWidth="1"/>
     <col min="8" max="9" width="35" style="4" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="31.5" style="37" customWidth="1"/>
-    <col min="11" max="11" width="19.83203125" style="36" customWidth="1"/>
-    <col min="12" max="13" width="20.5" style="38" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5" style="40" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5" style="38" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="31.5" style="36" customWidth="1"/>
+    <col min="11" max="11" width="19.83203125" style="35" customWidth="1"/>
+    <col min="12" max="14" width="20.5" style="37" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.5" style="38" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="37" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5" style="39" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" s="4" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="B1" s="42" t="s">
+      <c r="B1" s="40" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="5" t="s">
@@ -2091,7 +2086,9 @@
       <c r="M1" s="9" t="s">
         <v>406</v>
       </c>
-      <c r="N1" s="10"/>
+      <c r="N1" s="9" t="s">
+        <v>435</v>
+      </c>
       <c r="O1" s="10"/>
       <c r="P1" s="11"/>
       <c r="Q1" s="11"/>
@@ -2126,7 +2123,9 @@
       </c>
       <c r="L2" s="16"/>
       <c r="M2" s="16"/>
-      <c r="N2" s="10"/>
+      <c r="N2" s="16">
+        <v>1</v>
+      </c>
       <c r="O2" s="10"/>
       <c r="P2" s="11"/>
       <c r="Q2" s="11"/>
@@ -2135,7 +2134,7 @@
       <c r="A3" s="12" t="s">
         <v>208</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="41" t="s">
         <v>4</v>
       </c>
       <c r="C3" s="17" t="s">
@@ -2161,7 +2160,9 @@
       </c>
       <c r="L3" s="16"/>
       <c r="M3" s="16"/>
-      <c r="N3" s="10"/>
+      <c r="N3" s="16">
+        <v>1</v>
+      </c>
       <c r="O3" s="10"/>
       <c r="P3" s="11"/>
       <c r="Q3" s="11"/>
@@ -2196,7 +2197,9 @@
       </c>
       <c r="L4" s="16"/>
       <c r="M4" s="16"/>
-      <c r="N4" s="10"/>
+      <c r="N4" s="16">
+        <v>1</v>
+      </c>
       <c r="O4" s="10"/>
       <c r="P4" s="11"/>
       <c r="Q4" s="11"/>
@@ -2220,7 +2223,7 @@
       <c r="F5" s="12" t="s">
         <v>216</v>
       </c>
-      <c r="G5" s="48" t="s">
+      <c r="G5" s="46" t="s">
         <v>417</v>
       </c>
       <c r="H5" s="12"/>
@@ -2237,7 +2240,9 @@
       <c r="M5" s="16">
         <v>1</v>
       </c>
-      <c r="N5" s="10"/>
+      <c r="N5" s="16">
+        <v>1</v>
+      </c>
       <c r="O5" s="10"/>
       <c r="P5" s="11"/>
       <c r="Q5" s="11"/>
@@ -2276,7 +2281,7 @@
       </c>
       <c r="L6" s="16"/>
       <c r="M6" s="16"/>
-      <c r="N6" s="10"/>
+      <c r="N6" s="16"/>
       <c r="O6" s="10"/>
       <c r="P6" s="11"/>
       <c r="Q6" s="11"/>
@@ -2300,7 +2305,7 @@
       <c r="F7" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="G7" s="45" t="s">
+      <c r="G7" s="43" t="s">
         <v>416</v>
       </c>
       <c r="H7" s="12"/>
@@ -2312,10 +2317,12 @@
         <v>12</v>
       </c>
       <c r="L7" s="16"/>
-      <c r="M7" s="44">
-        <v>1</v>
-      </c>
-      <c r="N7" s="10"/>
+      <c r="M7" s="42">
+        <v>1</v>
+      </c>
+      <c r="N7" s="42">
+        <v>1</v>
+      </c>
       <c r="O7" s="10"/>
       <c r="P7" s="11"/>
       <c r="Q7" s="11"/>
@@ -2357,10 +2364,12 @@
       <c r="L8" s="16">
         <v>1</v>
       </c>
-      <c r="M8" s="44">
-        <v>1</v>
-      </c>
-      <c r="N8" s="10"/>
+      <c r="M8" s="42">
+        <v>1</v>
+      </c>
+      <c r="N8" s="16">
+        <v>1</v>
+      </c>
       <c r="O8" s="10"/>
       <c r="P8" s="11"/>
       <c r="Q8" s="11"/>
@@ -2398,8 +2407,10 @@
         <v>12</v>
       </c>
       <c r="L9" s="16"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="10"/>
+      <c r="M9" s="42"/>
+      <c r="N9" s="16">
+        <v>1</v>
+      </c>
       <c r="O9" s="10"/>
       <c r="P9" s="11"/>
       <c r="Q9" s="11"/>
@@ -2441,10 +2452,12 @@
       <c r="L10" s="16">
         <v>1</v>
       </c>
-      <c r="M10" s="44">
-        <v>1</v>
-      </c>
-      <c r="N10" s="10"/>
+      <c r="M10" s="42">
+        <v>1</v>
+      </c>
+      <c r="N10" s="16">
+        <v>1</v>
+      </c>
       <c r="O10" s="10"/>
       <c r="P10" s="11"/>
       <c r="Q10" s="11"/>
@@ -2478,8 +2491,10 @@
         <v>12</v>
       </c>
       <c r="L11" s="16"/>
-      <c r="M11" s="44"/>
-      <c r="N11" s="10"/>
+      <c r="M11" s="42"/>
+      <c r="N11" s="16">
+        <v>1</v>
+      </c>
       <c r="O11" s="10"/>
       <c r="P11" s="11"/>
       <c r="Q11" s="11"/>
@@ -2513,8 +2528,10 @@
         <v>12</v>
       </c>
       <c r="L12" s="16"/>
-      <c r="M12" s="44"/>
-      <c r="N12" s="10"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="16">
+        <v>1</v>
+      </c>
       <c r="O12" s="10"/>
       <c r="P12" s="11"/>
       <c r="Q12" s="11"/>
@@ -2556,10 +2573,12 @@
       <c r="L13" s="16">
         <v>1</v>
       </c>
-      <c r="M13" s="44">
-        <v>1</v>
-      </c>
-      <c r="N13" s="10"/>
+      <c r="M13" s="42">
+        <v>1</v>
+      </c>
+      <c r="N13" s="16">
+        <v>1</v>
+      </c>
       <c r="O13" s="10"/>
       <c r="P13" s="11"/>
       <c r="Q13" s="11"/>
@@ -2601,10 +2620,12 @@
       <c r="L14" s="16">
         <v>1</v>
       </c>
-      <c r="M14" s="44">
-        <v>1</v>
-      </c>
-      <c r="N14" s="10"/>
+      <c r="M14" s="42">
+        <v>1</v>
+      </c>
+      <c r="N14" s="16">
+        <v>1</v>
+      </c>
       <c r="O14" s="10"/>
       <c r="P14" s="11"/>
       <c r="Q14" s="11"/>
@@ -2640,10 +2661,12 @@
         <v>12</v>
       </c>
       <c r="L15" s="16"/>
-      <c r="M15" s="44">
-        <v>1</v>
-      </c>
-      <c r="N15" s="10"/>
+      <c r="M15" s="42">
+        <v>1</v>
+      </c>
+      <c r="N15" s="16">
+        <v>1</v>
+      </c>
       <c r="O15" s="10"/>
       <c r="P15" s="11"/>
       <c r="Q15" s="11"/>
@@ -2682,7 +2705,9 @@
       </c>
       <c r="L16" s="16"/>
       <c r="M16" s="16"/>
-      <c r="N16" s="10"/>
+      <c r="N16" s="16">
+        <v>1</v>
+      </c>
       <c r="O16" s="10"/>
       <c r="P16" s="11"/>
       <c r="Q16" s="11"/>
@@ -2721,7 +2746,9 @@
       </c>
       <c r="L17" s="16"/>
       <c r="M17" s="16"/>
-      <c r="N17" s="10"/>
+      <c r="N17" s="16">
+        <v>1</v>
+      </c>
       <c r="O17" s="10"/>
       <c r="P17" s="11"/>
       <c r="Q17" s="11"/>
@@ -2764,7 +2791,9 @@
       <c r="M18" s="16">
         <v>1</v>
       </c>
-      <c r="N18" s="10"/>
+      <c r="N18" s="16">
+        <v>1</v>
+      </c>
       <c r="O18" s="10"/>
       <c r="P18" s="11"/>
       <c r="Q18" s="11"/>
@@ -2799,7 +2828,9 @@
       </c>
       <c r="L19" s="16"/>
       <c r="M19" s="16"/>
-      <c r="N19" s="10"/>
+      <c r="N19" s="16">
+        <v>1</v>
+      </c>
       <c r="O19" s="10"/>
       <c r="P19" s="11"/>
       <c r="Q19" s="11"/>
@@ -2838,7 +2869,9 @@
       <c r="M20" s="16">
         <v>1</v>
       </c>
-      <c r="N20" s="10"/>
+      <c r="N20" s="16">
+        <v>1</v>
+      </c>
       <c r="O20" s="10"/>
       <c r="P20" s="11"/>
       <c r="Q20" s="11"/>
@@ -2877,7 +2910,9 @@
       <c r="M21" s="16">
         <v>1</v>
       </c>
-      <c r="N21" s="10"/>
+      <c r="N21" s="16">
+        <v>1</v>
+      </c>
       <c r="O21" s="10"/>
       <c r="P21" s="11"/>
       <c r="Q21" s="11"/>
@@ -2916,7 +2951,9 @@
       </c>
       <c r="L22" s="16"/>
       <c r="M22" s="16"/>
-      <c r="N22" s="10"/>
+      <c r="N22" s="16">
+        <v>3</v>
+      </c>
       <c r="O22" s="10"/>
       <c r="P22" s="11"/>
       <c r="Q22" s="11"/>
@@ -2959,7 +2996,9 @@
       <c r="M23" s="16">
         <v>1</v>
       </c>
-      <c r="N23" s="10"/>
+      <c r="N23" s="16">
+        <v>2</v>
+      </c>
       <c r="O23" s="10"/>
       <c r="P23" s="11"/>
       <c r="Q23" s="11"/>
@@ -3004,7 +3043,9 @@
       <c r="M24" s="16">
         <v>1</v>
       </c>
-      <c r="N24" s="10"/>
+      <c r="N24" s="16">
+        <v>3</v>
+      </c>
       <c r="O24" s="10"/>
       <c r="P24" s="11"/>
       <c r="Q24" s="11"/>
@@ -3043,7 +3084,9 @@
       </c>
       <c r="L25" s="16"/>
       <c r="M25" s="16"/>
-      <c r="N25" s="10"/>
+      <c r="N25" s="16">
+        <v>2</v>
+      </c>
       <c r="O25" s="10"/>
       <c r="P25" s="11"/>
       <c r="Q25" s="11"/>
@@ -3084,7 +3127,9 @@
       <c r="M26" s="16">
         <v>1</v>
       </c>
-      <c r="N26" s="28"/>
+      <c r="N26" s="16">
+        <v>2</v>
+      </c>
       <c r="O26" s="28"/>
       <c r="P26" s="29"/>
       <c r="Q26" s="30"/>
@@ -3125,7 +3170,9 @@
       <c r="M27" s="16">
         <v>1</v>
       </c>
-      <c r="N27" s="10"/>
+      <c r="N27" s="16">
+        <v>2</v>
+      </c>
       <c r="O27" s="10"/>
       <c r="P27" s="11"/>
       <c r="Q27" s="11"/>
@@ -3149,7 +3196,7 @@
       <c r="F28" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="G28" s="45" t="s">
+      <c r="G28" s="43" t="s">
         <v>418</v>
       </c>
       <c r="H28" s="12"/>
@@ -3166,7 +3213,9 @@
       <c r="M28" s="16">
         <v>1</v>
       </c>
-      <c r="N28" s="10"/>
+      <c r="N28" s="16">
+        <v>2</v>
+      </c>
       <c r="O28" s="10"/>
       <c r="P28" s="11"/>
       <c r="Q28" s="11"/>
@@ -3190,7 +3239,7 @@
       <c r="F29" s="12" t="s">
         <v>290</v>
       </c>
-      <c r="G29" s="45" t="s">
+      <c r="G29" s="43" t="s">
         <v>418</v>
       </c>
       <c r="H29" s="12"/>
@@ -3207,7 +3256,9 @@
       <c r="M29" s="16">
         <v>1</v>
       </c>
-      <c r="N29" s="10"/>
+      <c r="N29" s="16">
+        <v>2</v>
+      </c>
       <c r="O29" s="10"/>
       <c r="P29" s="11"/>
       <c r="Q29" s="11"/>
@@ -3234,21 +3285,23 @@
       <c r="G30" s="26" t="s">
         <v>432</v>
       </c>
-      <c r="H30" s="46"/>
-      <c r="I30" s="46"/>
+      <c r="H30" s="44"/>
+      <c r="I30" s="44"/>
       <c r="J30" s="15" t="s">
         <v>298</v>
       </c>
-      <c r="K30" s="49">
-        <v>12</v>
-      </c>
-      <c r="L30" s="47">
-        <v>1</v>
-      </c>
-      <c r="M30" s="47">
-        <v>1</v>
-      </c>
-      <c r="N30" s="10"/>
+      <c r="K30" s="47">
+        <v>12</v>
+      </c>
+      <c r="L30" s="45">
+        <v>1</v>
+      </c>
+      <c r="M30" s="45">
+        <v>1</v>
+      </c>
+      <c r="N30" s="16">
+        <v>2</v>
+      </c>
       <c r="O30" s="10"/>
       <c r="P30" s="11"/>
       <c r="Q30" s="11"/>
@@ -3283,7 +3336,9 @@
       </c>
       <c r="L31" s="16"/>
       <c r="M31" s="16"/>
-      <c r="N31" s="10"/>
+      <c r="N31" s="16">
+        <v>2</v>
+      </c>
       <c r="O31" s="10"/>
       <c r="P31" s="11"/>
       <c r="Q31" s="11"/>
@@ -3322,7 +3377,9 @@
       </c>
       <c r="L32" s="16"/>
       <c r="M32" s="16"/>
-      <c r="N32" s="31"/>
+      <c r="N32" s="16">
+        <v>2</v>
+      </c>
       <c r="O32" s="10"/>
       <c r="P32" s="11"/>
       <c r="Q32" s="11"/>
@@ -3359,7 +3416,9 @@
       </c>
       <c r="L33" s="16"/>
       <c r="M33" s="16"/>
-      <c r="N33" s="10"/>
+      <c r="N33" s="16">
+        <v>1</v>
+      </c>
       <c r="O33" s="10"/>
       <c r="P33" s="11"/>
       <c r="Q33" s="11"/>
@@ -3398,7 +3457,9 @@
       <c r="M34" s="16">
         <v>1</v>
       </c>
-      <c r="N34" s="10"/>
+      <c r="N34" s="16">
+        <v>1</v>
+      </c>
       <c r="O34" s="10"/>
       <c r="P34" s="11"/>
       <c r="Q34" s="11"/>
@@ -3432,8 +3493,10 @@
         <v>12</v>
       </c>
       <c r="L35" s="16"/>
-      <c r="M35" s="44"/>
-      <c r="N35" s="10"/>
+      <c r="M35" s="42"/>
+      <c r="N35" s="16">
+        <v>1</v>
+      </c>
       <c r="O35" s="10"/>
       <c r="P35" s="11"/>
       <c r="Q35" s="11"/>
@@ -3471,10 +3534,12 @@
       <c r="L36" s="16">
         <v>1</v>
       </c>
-      <c r="M36" s="44">
-        <v>1</v>
-      </c>
-      <c r="N36" s="10"/>
+      <c r="M36" s="42">
+        <v>1</v>
+      </c>
+      <c r="N36" s="16">
+        <v>1</v>
+      </c>
       <c r="O36" s="10"/>
       <c r="P36" s="11"/>
       <c r="Q36" s="11"/>
@@ -3512,10 +3577,12 @@
       <c r="L37" s="16">
         <v>1</v>
       </c>
-      <c r="M37" s="44">
-        <v>1</v>
-      </c>
-      <c r="N37" s="10"/>
+      <c r="M37" s="42">
+        <v>1</v>
+      </c>
+      <c r="N37" s="16">
+        <v>1</v>
+      </c>
       <c r="O37" s="10"/>
       <c r="P37" s="11"/>
       <c r="Q37" s="11"/>
@@ -3550,7 +3617,7 @@
       </c>
       <c r="L38" s="16"/>
       <c r="M38" s="16"/>
-      <c r="N38" s="10"/>
+      <c r="N38" s="16"/>
       <c r="O38" s="10"/>
       <c r="P38" s="11"/>
       <c r="Q38" s="11"/>
@@ -3589,7 +3656,9 @@
       <c r="M39" s="16">
         <v>1</v>
       </c>
-      <c r="N39" s="10"/>
+      <c r="N39" s="16">
+        <v>1</v>
+      </c>
       <c r="O39" s="10"/>
       <c r="P39" s="11"/>
       <c r="Q39" s="11"/>
@@ -3631,10 +3700,12 @@
       <c r="L40" s="16">
         <v>1</v>
       </c>
-      <c r="M40" s="44">
-        <v>1</v>
-      </c>
-      <c r="N40" s="10"/>
+      <c r="M40" s="42">
+        <v>1</v>
+      </c>
+      <c r="N40" s="16">
+        <v>1</v>
+      </c>
       <c r="O40" s="10"/>
       <c r="P40" s="11"/>
       <c r="Q40" s="11"/>
@@ -3672,8 +3743,10 @@
         <v>12</v>
       </c>
       <c r="L41" s="16"/>
-      <c r="M41" s="44"/>
-      <c r="N41" s="10"/>
+      <c r="M41" s="42"/>
+      <c r="N41" s="16">
+        <v>2</v>
+      </c>
       <c r="O41" s="10"/>
       <c r="P41" s="11"/>
       <c r="Q41" s="11"/>
@@ -3711,8 +3784,10 @@
         <v>12</v>
       </c>
       <c r="L42" s="16"/>
-      <c r="M42" s="44"/>
-      <c r="N42" s="10"/>
+      <c r="M42" s="42"/>
+      <c r="N42" s="16">
+        <v>2</v>
+      </c>
       <c r="O42" s="10"/>
       <c r="P42" s="11"/>
       <c r="Q42" s="11"/>
@@ -3746,8 +3821,10 @@
         <v>12</v>
       </c>
       <c r="L43" s="16"/>
-      <c r="M43" s="44"/>
-      <c r="N43" s="10"/>
+      <c r="M43" s="42"/>
+      <c r="N43" s="16">
+        <v>2</v>
+      </c>
       <c r="O43" s="10"/>
       <c r="P43" s="11"/>
       <c r="Q43" s="11"/>
@@ -3785,10 +3862,12 @@
       <c r="L44" s="16">
         <v>1</v>
       </c>
-      <c r="M44" s="44">
+      <c r="M44" s="42">
         <v>1.2</v>
       </c>
-      <c r="N44" s="10"/>
+      <c r="N44" s="16">
+        <v>1</v>
+      </c>
       <c r="O44" s="10"/>
       <c r="P44" s="11"/>
       <c r="Q44" s="11"/>
@@ -3830,10 +3909,12 @@
       <c r="L45" s="16">
         <v>1</v>
       </c>
-      <c r="M45" s="44">
+      <c r="M45" s="42">
         <v>1.2</v>
       </c>
-      <c r="N45" s="10"/>
+      <c r="N45" s="16">
+        <v>1</v>
+      </c>
       <c r="O45" s="10"/>
       <c r="P45" s="11"/>
       <c r="Q45" s="11"/>
@@ -3875,10 +3956,12 @@
       <c r="L46" s="16">
         <v>1</v>
       </c>
-      <c r="M46" s="44">
+      <c r="M46" s="42">
         <v>1.2</v>
       </c>
-      <c r="N46" s="10"/>
+      <c r="N46" s="16">
+        <v>1</v>
+      </c>
       <c r="O46" s="10"/>
       <c r="P46" s="11"/>
       <c r="Q46" s="11"/>
@@ -3916,10 +3999,12 @@
       <c r="L47" s="16">
         <v>1</v>
       </c>
-      <c r="M47" s="44">
+      <c r="M47" s="42">
         <v>1.2</v>
       </c>
-      <c r="N47" s="10"/>
+      <c r="N47" s="16">
+        <v>1</v>
+      </c>
       <c r="O47" s="10"/>
       <c r="P47" s="11"/>
       <c r="Q47" s="11"/>
@@ -3959,10 +4044,12 @@
         <v>12</v>
       </c>
       <c r="L48" s="16"/>
-      <c r="M48" s="44">
-        <v>1</v>
-      </c>
-      <c r="N48" s="10"/>
+      <c r="M48" s="42">
+        <v>1</v>
+      </c>
+      <c r="N48" s="16">
+        <v>1</v>
+      </c>
       <c r="O48" s="10"/>
       <c r="P48" s="11"/>
       <c r="Q48" s="11"/>
@@ -4004,10 +4091,12 @@
       <c r="L49" s="16">
         <v>1</v>
       </c>
-      <c r="M49" s="44">
-        <v>1</v>
-      </c>
-      <c r="N49" s="10"/>
+      <c r="M49" s="42">
+        <v>1</v>
+      </c>
+      <c r="N49" s="16">
+        <v>1</v>
+      </c>
       <c r="O49" s="10"/>
       <c r="P49" s="11"/>
       <c r="Q49" s="11"/>
@@ -4047,10 +4136,12 @@
         <v>12</v>
       </c>
       <c r="L50" s="16"/>
-      <c r="M50" s="44">
-        <v>1</v>
-      </c>
-      <c r="N50" s="10"/>
+      <c r="M50" s="42">
+        <v>1</v>
+      </c>
+      <c r="N50" s="16">
+        <v>1</v>
+      </c>
       <c r="O50" s="10"/>
       <c r="P50" s="11"/>
       <c r="Q50" s="11"/>
@@ -4085,7 +4176,9 @@
       </c>
       <c r="L51" s="16"/>
       <c r="M51" s="16"/>
-      <c r="N51" s="10"/>
+      <c r="N51" s="16">
+        <v>1</v>
+      </c>
       <c r="O51" s="10"/>
       <c r="P51" s="11"/>
       <c r="Q51" s="11"/>
@@ -4124,7 +4217,7 @@
       </c>
       <c r="L52" s="16"/>
       <c r="M52" s="16"/>
-      <c r="N52" s="10"/>
+      <c r="N52" s="16"/>
       <c r="O52" s="10"/>
       <c r="P52" s="11"/>
       <c r="Q52" s="11"/>
@@ -4163,7 +4256,9 @@
       </c>
       <c r="L53" s="16"/>
       <c r="M53" s="16"/>
-      <c r="N53" s="10"/>
+      <c r="N53" s="16">
+        <v>2</v>
+      </c>
       <c r="O53" s="10"/>
       <c r="P53" s="11"/>
       <c r="Q53" s="11"/>
@@ -4202,7 +4297,9 @@
       </c>
       <c r="L54" s="16"/>
       <c r="M54" s="16"/>
-      <c r="N54" s="10"/>
+      <c r="N54" s="16">
+        <v>2</v>
+      </c>
       <c r="O54" s="10"/>
       <c r="P54" s="11"/>
       <c r="Q54" s="11"/>
@@ -4241,7 +4338,9 @@
       </c>
       <c r="L55" s="16"/>
       <c r="M55" s="16"/>
-      <c r="N55" s="10"/>
+      <c r="N55" s="16">
+        <v>2</v>
+      </c>
       <c r="O55" s="10"/>
       <c r="P55" s="11"/>
       <c r="Q55" s="11"/>
@@ -4286,7 +4385,9 @@
       <c r="M56" s="16">
         <v>1</v>
       </c>
-      <c r="N56" s="10"/>
+      <c r="N56" s="16">
+        <v>2</v>
+      </c>
       <c r="O56" s="10"/>
       <c r="P56" s="11"/>
       <c r="Q56" s="11"/>
@@ -4327,7 +4428,9 @@
       <c r="M57" s="16">
         <v>1</v>
       </c>
-      <c r="N57" s="10"/>
+      <c r="N57" s="16">
+        <v>2</v>
+      </c>
       <c r="O57" s="10"/>
       <c r="P57" s="11"/>
       <c r="Q57" s="11"/>
@@ -4372,7 +4475,9 @@
       <c r="M58" s="16">
         <v>1</v>
       </c>
-      <c r="N58" s="10"/>
+      <c r="N58" s="16">
+        <v>2</v>
+      </c>
       <c r="O58" s="10"/>
       <c r="P58" s="11"/>
       <c r="Q58" s="11"/>
@@ -4399,21 +4504,23 @@
       <c r="G59" s="26" t="s">
         <v>433</v>
       </c>
-      <c r="H59" s="46"/>
-      <c r="I59" s="46"/>
+      <c r="H59" s="44"/>
+      <c r="I59" s="44"/>
       <c r="J59" s="15">
         <v>0.85</v>
       </c>
-      <c r="K59" s="49">
-        <v>12</v>
-      </c>
-      <c r="L59" s="47">
-        <v>1</v>
-      </c>
-      <c r="M59" s="47">
-        <v>1</v>
-      </c>
-      <c r="N59" s="10"/>
+      <c r="K59" s="47">
+        <v>12</v>
+      </c>
+      <c r="L59" s="45">
+        <v>1</v>
+      </c>
+      <c r="M59" s="45">
+        <v>1</v>
+      </c>
+      <c r="N59" s="16">
+        <v>2</v>
+      </c>
       <c r="O59" s="31"/>
       <c r="P59" s="29"/>
       <c r="Q59" s="30"/>
@@ -4456,7 +4563,9 @@
       <c r="M60" s="16">
         <v>1</v>
       </c>
-      <c r="N60" s="10"/>
+      <c r="N60" s="16">
+        <v>2</v>
+      </c>
       <c r="O60" s="31"/>
       <c r="P60" s="29"/>
       <c r="Q60" s="30"/>
@@ -4497,7 +4606,9 @@
       </c>
       <c r="L61" s="16"/>
       <c r="M61" s="16"/>
-      <c r="N61" s="10"/>
+      <c r="N61" s="16">
+        <v>2</v>
+      </c>
       <c r="O61" s="31"/>
       <c r="P61" s="29"/>
       <c r="Q61" s="28"/>
@@ -4544,10 +4655,12 @@
       <c r="M62" s="16">
         <v>1</v>
       </c>
-      <c r="N62" s="10"/>
-      <c r="O62" s="40"/>
-      <c r="P62" s="38"/>
-      <c r="Q62" s="41"/>
+      <c r="N62" s="16">
+        <v>2</v>
+      </c>
+      <c r="O62" s="38"/>
+      <c r="P62" s="37"/>
+      <c r="Q62" s="39"/>
       <c r="R62"/>
       <c r="S62"/>
     </row>
@@ -4565,7 +4678,7 @@
       <c r="K63" s="33"/>
       <c r="L63" s="29"/>
       <c r="M63" s="29"/>
-      <c r="N63" s="31"/>
+      <c r="N63" s="29"/>
     </row>
     <row r="64" spans="1:19" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="19"/>
@@ -4581,7 +4694,7 @@
       <c r="K64" s="33"/>
       <c r="L64" s="29"/>
       <c r="M64" s="29"/>
-      <c r="N64" s="31"/>
+      <c r="N64" s="29"/>
     </row>
     <row r="65" spans="1:14" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="19"/>
@@ -4597,12 +4710,36 @@
       <c r="K65" s="33"/>
       <c r="L65" s="29"/>
       <c r="M65" s="29"/>
-      <c r="N65" s="35"/>
+      <c r="N65" s="29"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M62" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="C1:N65" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="L1:M1048576">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L1:N1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N1:N1048576">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
update strategies for bulgaria by matching the WEM and WAM strategies to the NECP targets
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_wem_wam.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_bulgaria_transformation_wem_wam.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tony/Documents/sisepuede_modeling/ssp_bulgaria/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14864F2C-0BC5-D444-B08F-047A4EE7BF0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83436267-B02C-314C-834D-D3E20A1E466E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36700" yWindow="2860" windowWidth="32100" windowHeight="19840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4080" yWindow="500" windowWidth="30240" windowHeight="17720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>

</xml_diff>